<commit_message>
Ajout du bouton de lancement de veille dans le dashboard
</commit_message>
<xml_diff>
--- a/docs/dossiers/dossier-asnieres-sur-seine-c20580d4.xlsx
+++ b/docs/dossiers/dossier-asnieres-sur-seine-c20580d4.xlsx
@@ -833,7 +833,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>Dossier généré le 06/08/2026 — indicatif, l'offre de prêt de la banque fait foi.</t>
+          <t>Dossier généré le 07/08/2026 — indicatif, l'offre de prêt de la banque fait foi.</t>
         </is>
       </c>
     </row>
@@ -929,7 +929,7 @@
     <row r="13">
       <c r="A13" s="13" t="inlineStr">
         <is>
-          <t>EN CLAIR — Sur la base d'un loyer ESTIMÉ (pas de bail signé à ce stade) : aux hypothèses de ce dossier (apport 20 %, crédit 4,58 % sur 20 ans, charges provisionnées), le bien s'autofinance : le loyer couvre crédit et charges et laisse environ +66 €/mois.</t>
+          <t>EN CLAIR — Sur la base d'un loyer ESTIMÉ (pas de bail signé à ce stade) : aux hypothèses de ce dossier (apport 20 %, crédit 3,9 % sur 20 ans, charges provisionnées), le bien s'autofinance : le loyer couvre crédit et charges et laisse environ +169 €/mois.</t>
         </is>
       </c>
     </row>
@@ -1082,7 +1082,7 @@
         </is>
       </c>
       <c r="B28" s="20" t="n">
-        <v>0.0458</v>
+        <v>0.039</v>
       </c>
     </row>
     <row r="29">

</xml_diff>